<commit_message>
Update galpones dashboard data
</commit_message>
<xml_diff>
--- a/data/galpones/informe_galpones.xlsx
+++ b/data/galpones/informe_galpones.xlsx
@@ -25,7 +25,7 @@
     <t>Desde: 01/01/2026</t>
   </si>
   <si>
-    <t>Hasta: 08/05/2026</t>
+    <t>Hasta: 09/05/2026</t>
   </si>
   <si>
     <t>Fecha</t>
@@ -2155,28 +2155,28 @@
         <v>15</v>
       </c>
       <c r="C41">
-        <v>20089</v>
+        <v>8763</v>
       </c>
       <c r="D41">
-        <v>71.0</v>
+        <v>40.0</v>
       </c>
       <c r="E41">
-        <v>14612</v>
+        <v>7680</v>
       </c>
       <c r="F41">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="G41">
-        <v>72.74</v>
+        <v>87.64</v>
       </c>
       <c r="H41">
-        <v>88.36</v>
+        <v>114.12</v>
       </c>
       <c r="I41">
-        <v>35.0</v>
+        <v>33.0</v>
       </c>
       <c r="J41">
-        <v>3082.0</v>
+        <v>2000.0</v>
       </c>
       <c r="K41"/>
     </row>
@@ -2188,28 +2188,28 @@
         <v>15</v>
       </c>
       <c r="C42">
-        <v>8763</v>
+        <v>20089</v>
       </c>
       <c r="D42">
-        <v>40.0</v>
+        <v>71.0</v>
       </c>
       <c r="E42">
-        <v>7680</v>
+        <v>14612</v>
       </c>
       <c r="F42">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="G42">
-        <v>87.64</v>
+        <v>72.74</v>
       </c>
       <c r="H42">
-        <v>114.12</v>
+        <v>88.36</v>
       </c>
       <c r="I42">
-        <v>33.0</v>
+        <v>35.0</v>
       </c>
       <c r="J42">
-        <v>2000.0</v>
+        <v>3082.0</v>
       </c>
       <c r="K42"/>
     </row>
@@ -3683,28 +3683,28 @@
         <v>15</v>
       </c>
       <c r="C87">
-        <v>8502</v>
+        <v>8508</v>
       </c>
       <c r="D87">
         <v>40.0</v>
       </c>
       <c r="E87">
-        <v>7208</v>
+        <v>7272</v>
       </c>
       <c r="F87">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G87">
-        <v>84.78</v>
+        <v>85.47</v>
       </c>
       <c r="H87">
-        <v>117.62</v>
+        <v>117.54</v>
       </c>
       <c r="I87">
-        <v>33.0</v>
+        <v>31.0</v>
       </c>
       <c r="J87">
-        <v>2000.0</v>
+        <v>2200.0</v>
       </c>
       <c r="K87"/>
     </row>
@@ -3716,28 +3716,28 @@
         <v>15</v>
       </c>
       <c r="C88">
-        <v>8508</v>
+        <v>8502</v>
       </c>
       <c r="D88">
         <v>40.0</v>
       </c>
       <c r="E88">
-        <v>7272</v>
+        <v>7208</v>
       </c>
       <c r="F88">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G88">
-        <v>85.47</v>
+        <v>84.78</v>
       </c>
       <c r="H88">
-        <v>117.54</v>
+        <v>117.62</v>
       </c>
       <c r="I88">
-        <v>31.0</v>
+        <v>33.0</v>
       </c>
       <c r="J88">
-        <v>2200.0</v>
+        <v>2000.0</v>
       </c>
       <c r="K88"/>
     </row>

</xml_diff>